<commit_message>
Update university branding, address, login header style, and label 'Admin' to 'Akademik'
</commit_message>
<xml_diff>
--- a/dummy_mahasiswa_terbaru.xlsx
+++ b/dummy_mahasiswa_terbaru.xlsx
@@ -1,27 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\XPROJECT\x6\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4CA63C-3F07-4FC2-8661-6CE24E4D92FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Data Mahasiswa" sheetId="1" r:id="rId1"/>
-    <sheet name="Referensi" sheetId="2" r:id="rId2"/>
+    <sheet name="Data Mahasiswa" sheetId="1" r:id="rId4"/>
+    <sheet name="Referensi" sheetId="2" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="34">
   <si>
     <t>nim*</t>
   </si>
@@ -71,15 +66,24 @@
     <t>nomor_ijazah</t>
   </si>
   <si>
+    <t>Nama Mahasiswa 37</t>
+  </si>
+  <si>
     <t>Pembangunan Sosial</t>
   </si>
   <si>
+    <t>215100037@unida-aceh.ac.id</t>
+  </si>
+  <si>
     <t>Laki-laki</t>
   </si>
   <si>
     <t>Islam</t>
   </si>
   <si>
+    <t>Jl. Contoh Alamat</t>
+  </si>
+  <si>
     <t>2021-08-01</t>
   </si>
   <si>
@@ -114,31 +118,21 @@
   </si>
   <si>
     <t>Mengundurkan Diri</t>
-  </si>
-  <si>
-    <t>2029170123@unida-aceh.ac.id</t>
-  </si>
-  <si>
-    <t>Nama Mahasiswa</t>
-  </si>
-  <si>
-    <t>Desa. Mibo, Jalan. Utama, Nomor 22, KecamatanBanda Raya, Banda Aceh</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -159,28 +153,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+  <cellXfs count="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -470,19 +453,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.54296875" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.36328125" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:P100"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -532,30 +510,30 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16">
       <c r="A2">
-        <v>2029170123</v>
+        <v>215100037</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>31</v>
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
       </c>
       <c r="E2">
-        <v>1171010101900000</v>
+        <v>1234567890123037</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="I2">
         <v>2021</v>
@@ -564,107 +542,800 @@
         <v>2021</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="N2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="O2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="P2" t="s">
-        <v>24</v>
-      </c>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="C3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="L3"/>
+      <c r="O3"/>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="C4"/>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="L4"/>
+      <c r="O4"/>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="C5"/>
+      <c r="F5"/>
+      <c r="G5"/>
+      <c r="L5"/>
+      <c r="O5"/>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="C6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="L6"/>
+      <c r="O6"/>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="C7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="L7"/>
+      <c r="O7"/>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="C8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="L8"/>
+      <c r="O8"/>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="C9"/>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="L9"/>
+      <c r="O9"/>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="C10"/>
+      <c r="F10"/>
+      <c r="G10"/>
+      <c r="L10"/>
+      <c r="O10"/>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="C11"/>
+      <c r="F11"/>
+      <c r="G11"/>
+      <c r="L11"/>
+      <c r="O11"/>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="C12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+      <c r="L12"/>
+      <c r="O12"/>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="C13"/>
+      <c r="F13"/>
+      <c r="G13"/>
+      <c r="L13"/>
+      <c r="O13"/>
+    </row>
+    <row r="14" spans="1:16">
+      <c r="C14"/>
+      <c r="F14"/>
+      <c r="G14"/>
+      <c r="L14"/>
+      <c r="O14"/>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="C15"/>
+      <c r="F15"/>
+      <c r="G15"/>
+      <c r="L15"/>
+      <c r="O15"/>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="C16"/>
+      <c r="F16"/>
+      <c r="G16"/>
+      <c r="L16"/>
+      <c r="O16"/>
+    </row>
+    <row r="17" spans="1:16">
+      <c r="C17"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="L17"/>
+      <c r="O17"/>
+    </row>
+    <row r="18" spans="1:16">
+      <c r="C18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="L18"/>
+      <c r="O18"/>
+    </row>
+    <row r="19" spans="1:16">
+      <c r="C19"/>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="L19"/>
+      <c r="O19"/>
+    </row>
+    <row r="20" spans="1:16">
+      <c r="C20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="L20"/>
+      <c r="O20"/>
+    </row>
+    <row r="21" spans="1:16">
+      <c r="C21"/>
+      <c r="F21"/>
+      <c r="G21"/>
+      <c r="L21"/>
+      <c r="O21"/>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="C22"/>
+      <c r="F22"/>
+      <c r="G22"/>
+      <c r="L22"/>
+      <c r="O22"/>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="C23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="L23"/>
+      <c r="O23"/>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="C24"/>
+      <c r="F24"/>
+      <c r="G24"/>
+      <c r="L24"/>
+      <c r="O24"/>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="C25"/>
+      <c r="F25"/>
+      <c r="G25"/>
+      <c r="L25"/>
+      <c r="O25"/>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="C26"/>
+      <c r="F26"/>
+      <c r="G26"/>
+      <c r="L26"/>
+      <c r="O26"/>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="C27"/>
+      <c r="F27"/>
+      <c r="G27"/>
+      <c r="L27"/>
+      <c r="O27"/>
+    </row>
+    <row r="28" spans="1:16">
+      <c r="C28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="L28"/>
+      <c r="O28"/>
+    </row>
+    <row r="29" spans="1:16">
+      <c r="C29"/>
+      <c r="F29"/>
+      <c r="G29"/>
+      <c r="L29"/>
+      <c r="O29"/>
+    </row>
+    <row r="30" spans="1:16">
+      <c r="C30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="L30"/>
+      <c r="O30"/>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="C31"/>
+      <c r="F31"/>
+      <c r="G31"/>
+      <c r="L31"/>
+      <c r="O31"/>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="C32"/>
+      <c r="F32"/>
+      <c r="G32"/>
+      <c r="L32"/>
+      <c r="O32"/>
+    </row>
+    <row r="33" spans="1:16">
+      <c r="C33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="L33"/>
+      <c r="O33"/>
+    </row>
+    <row r="34" spans="1:16">
+      <c r="C34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="L34"/>
+      <c r="O34"/>
+    </row>
+    <row r="35" spans="1:16">
+      <c r="C35"/>
+      <c r="F35"/>
+      <c r="G35"/>
+      <c r="L35"/>
+      <c r="O35"/>
+    </row>
+    <row r="36" spans="1:16">
+      <c r="C36"/>
+      <c r="F36"/>
+      <c r="G36"/>
+      <c r="L36"/>
+      <c r="O36"/>
+    </row>
+    <row r="37" spans="1:16">
+      <c r="C37"/>
+      <c r="F37"/>
+      <c r="G37"/>
+      <c r="L37"/>
+      <c r="O37"/>
+    </row>
+    <row r="38" spans="1:16">
+      <c r="C38"/>
+      <c r="F38"/>
+      <c r="G38"/>
+      <c r="L38"/>
+      <c r="O38"/>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="C39"/>
+      <c r="F39"/>
+      <c r="G39"/>
+      <c r="L39"/>
+      <c r="O39"/>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="C40"/>
+      <c r="F40"/>
+      <c r="G40"/>
+      <c r="L40"/>
+      <c r="O40"/>
+    </row>
+    <row r="41" spans="1:16">
+      <c r="C41"/>
+      <c r="F41"/>
+      <c r="G41"/>
+      <c r="L41"/>
+      <c r="O41"/>
+    </row>
+    <row r="42" spans="1:16">
+      <c r="C42"/>
+      <c r="F42"/>
+      <c r="G42"/>
+      <c r="L42"/>
+      <c r="O42"/>
+    </row>
+    <row r="43" spans="1:16">
+      <c r="C43"/>
+      <c r="F43"/>
+      <c r="G43"/>
+      <c r="L43"/>
+      <c r="O43"/>
+    </row>
+    <row r="44" spans="1:16">
+      <c r="C44"/>
+      <c r="F44"/>
+      <c r="G44"/>
+      <c r="L44"/>
+      <c r="O44"/>
+    </row>
+    <row r="45" spans="1:16">
+      <c r="C45"/>
+      <c r="F45"/>
+      <c r="G45"/>
+      <c r="L45"/>
+      <c r="O45"/>
+    </row>
+    <row r="46" spans="1:16">
+      <c r="C46"/>
+      <c r="F46"/>
+      <c r="G46"/>
+      <c r="L46"/>
+      <c r="O46"/>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="C47"/>
+      <c r="F47"/>
+      <c r="G47"/>
+      <c r="L47"/>
+      <c r="O47"/>
+    </row>
+    <row r="48" spans="1:16">
+      <c r="C48"/>
+      <c r="F48"/>
+      <c r="G48"/>
+      <c r="L48"/>
+      <c r="O48"/>
+    </row>
+    <row r="49" spans="1:16">
+      <c r="C49"/>
+      <c r="F49"/>
+      <c r="G49"/>
+      <c r="L49"/>
+      <c r="O49"/>
+    </row>
+    <row r="50" spans="1:16">
+      <c r="C50"/>
+      <c r="F50"/>
+      <c r="G50"/>
+      <c r="L50"/>
+      <c r="O50"/>
+    </row>
+    <row r="51" spans="1:16">
+      <c r="C51"/>
+      <c r="F51"/>
+      <c r="G51"/>
+      <c r="L51"/>
+      <c r="O51"/>
+    </row>
+    <row r="52" spans="1:16">
+      <c r="C52"/>
+      <c r="F52"/>
+      <c r="G52"/>
+      <c r="L52"/>
+      <c r="O52"/>
+    </row>
+    <row r="53" spans="1:16">
+      <c r="C53"/>
+      <c r="F53"/>
+      <c r="G53"/>
+      <c r="L53"/>
+      <c r="O53"/>
+    </row>
+    <row r="54" spans="1:16">
+      <c r="C54"/>
+      <c r="F54"/>
+      <c r="G54"/>
+      <c r="L54"/>
+      <c r="O54"/>
+    </row>
+    <row r="55" spans="1:16">
+      <c r="C55"/>
+      <c r="F55"/>
+      <c r="G55"/>
+      <c r="L55"/>
+      <c r="O55"/>
+    </row>
+    <row r="56" spans="1:16">
+      <c r="C56"/>
+      <c r="F56"/>
+      <c r="G56"/>
+      <c r="L56"/>
+      <c r="O56"/>
+    </row>
+    <row r="57" spans="1:16">
+      <c r="C57"/>
+      <c r="F57"/>
+      <c r="G57"/>
+      <c r="L57"/>
+      <c r="O57"/>
+    </row>
+    <row r="58" spans="1:16">
+      <c r="C58"/>
+      <c r="F58"/>
+      <c r="G58"/>
+      <c r="L58"/>
+      <c r="O58"/>
+    </row>
+    <row r="59" spans="1:16">
+      <c r="C59"/>
+      <c r="F59"/>
+      <c r="G59"/>
+      <c r="L59"/>
+      <c r="O59"/>
+    </row>
+    <row r="60" spans="1:16">
+      <c r="C60"/>
+      <c r="F60"/>
+      <c r="G60"/>
+      <c r="L60"/>
+      <c r="O60"/>
+    </row>
+    <row r="61" spans="1:16">
+      <c r="C61"/>
+      <c r="F61"/>
+      <c r="G61"/>
+      <c r="L61"/>
+      <c r="O61"/>
+    </row>
+    <row r="62" spans="1:16">
+      <c r="C62"/>
+      <c r="F62"/>
+      <c r="G62"/>
+      <c r="L62"/>
+      <c r="O62"/>
+    </row>
+    <row r="63" spans="1:16">
+      <c r="C63"/>
+      <c r="F63"/>
+      <c r="G63"/>
+      <c r="L63"/>
+      <c r="O63"/>
+    </row>
+    <row r="64" spans="1:16">
+      <c r="C64"/>
+      <c r="F64"/>
+      <c r="G64"/>
+      <c r="L64"/>
+      <c r="O64"/>
+    </row>
+    <row r="65" spans="1:16">
+      <c r="C65"/>
+      <c r="F65"/>
+      <c r="G65"/>
+      <c r="L65"/>
+      <c r="O65"/>
+    </row>
+    <row r="66" spans="1:16">
+      <c r="C66"/>
+      <c r="F66"/>
+      <c r="G66"/>
+      <c r="L66"/>
+      <c r="O66"/>
+    </row>
+    <row r="67" spans="1:16">
+      <c r="C67"/>
+      <c r="F67"/>
+      <c r="G67"/>
+      <c r="L67"/>
+      <c r="O67"/>
+    </row>
+    <row r="68" spans="1:16">
+      <c r="C68"/>
+      <c r="F68"/>
+      <c r="G68"/>
+      <c r="L68"/>
+      <c r="O68"/>
+    </row>
+    <row r="69" spans="1:16">
+      <c r="C69"/>
+      <c r="F69"/>
+      <c r="G69"/>
+      <c r="L69"/>
+      <c r="O69"/>
+    </row>
+    <row r="70" spans="1:16">
+      <c r="C70"/>
+      <c r="F70"/>
+      <c r="G70"/>
+      <c r="L70"/>
+      <c r="O70"/>
+    </row>
+    <row r="71" spans="1:16">
+      <c r="C71"/>
+      <c r="F71"/>
+      <c r="G71"/>
+      <c r="L71"/>
+      <c r="O71"/>
+    </row>
+    <row r="72" spans="1:16">
+      <c r="C72"/>
+      <c r="F72"/>
+      <c r="G72"/>
+      <c r="L72"/>
+      <c r="O72"/>
+    </row>
+    <row r="73" spans="1:16">
+      <c r="C73"/>
+      <c r="F73"/>
+      <c r="G73"/>
+      <c r="L73"/>
+      <c r="O73"/>
+    </row>
+    <row r="74" spans="1:16">
+      <c r="C74"/>
+      <c r="F74"/>
+      <c r="G74"/>
+      <c r="L74"/>
+      <c r="O74"/>
+    </row>
+    <row r="75" spans="1:16">
+      <c r="C75"/>
+      <c r="F75"/>
+      <c r="G75"/>
+      <c r="L75"/>
+      <c r="O75"/>
+    </row>
+    <row r="76" spans="1:16">
+      <c r="C76"/>
+      <c r="F76"/>
+      <c r="G76"/>
+      <c r="L76"/>
+      <c r="O76"/>
+    </row>
+    <row r="77" spans="1:16">
+      <c r="C77"/>
+      <c r="F77"/>
+      <c r="G77"/>
+      <c r="L77"/>
+      <c r="O77"/>
+    </row>
+    <row r="78" spans="1:16">
+      <c r="C78"/>
+      <c r="F78"/>
+      <c r="G78"/>
+      <c r="L78"/>
+      <c r="O78"/>
+    </row>
+    <row r="79" spans="1:16">
+      <c r="C79"/>
+      <c r="F79"/>
+      <c r="G79"/>
+      <c r="L79"/>
+      <c r="O79"/>
+    </row>
+    <row r="80" spans="1:16">
+      <c r="C80"/>
+      <c r="F80"/>
+      <c r="G80"/>
+      <c r="L80"/>
+      <c r="O80"/>
+    </row>
+    <row r="81" spans="1:16">
+      <c r="C81"/>
+      <c r="F81"/>
+      <c r="G81"/>
+      <c r="L81"/>
+      <c r="O81"/>
+    </row>
+    <row r="82" spans="1:16">
+      <c r="C82"/>
+      <c r="F82"/>
+      <c r="G82"/>
+      <c r="L82"/>
+      <c r="O82"/>
+    </row>
+    <row r="83" spans="1:16">
+      <c r="C83"/>
+      <c r="F83"/>
+      <c r="G83"/>
+      <c r="L83"/>
+      <c r="O83"/>
+    </row>
+    <row r="84" spans="1:16">
+      <c r="C84"/>
+      <c r="F84"/>
+      <c r="G84"/>
+      <c r="L84"/>
+      <c r="O84"/>
+    </row>
+    <row r="85" spans="1:16">
+      <c r="C85"/>
+      <c r="F85"/>
+      <c r="G85"/>
+      <c r="L85"/>
+      <c r="O85"/>
+    </row>
+    <row r="86" spans="1:16">
+      <c r="C86"/>
+      <c r="F86"/>
+      <c r="G86"/>
+      <c r="L86"/>
+      <c r="O86"/>
+    </row>
+    <row r="87" spans="1:16">
+      <c r="C87"/>
+      <c r="F87"/>
+      <c r="G87"/>
+      <c r="L87"/>
+      <c r="O87"/>
+    </row>
+    <row r="88" spans="1:16">
+      <c r="C88"/>
+      <c r="F88"/>
+      <c r="G88"/>
+      <c r="L88"/>
+      <c r="O88"/>
+    </row>
+    <row r="89" spans="1:16">
+      <c r="C89"/>
+      <c r="F89"/>
+      <c r="G89"/>
+      <c r="L89"/>
+      <c r="O89"/>
+    </row>
+    <row r="90" spans="1:16">
+      <c r="C90"/>
+      <c r="F90"/>
+      <c r="G90"/>
+      <c r="L90"/>
+      <c r="O90"/>
+    </row>
+    <row r="91" spans="1:16">
+      <c r="C91"/>
+      <c r="F91"/>
+      <c r="G91"/>
+      <c r="L91"/>
+      <c r="O91"/>
+    </row>
+    <row r="92" spans="1:16">
+      <c r="C92"/>
+      <c r="F92"/>
+      <c r="G92"/>
+      <c r="L92"/>
+      <c r="O92"/>
+    </row>
+    <row r="93" spans="1:16">
+      <c r="C93"/>
+      <c r="F93"/>
+      <c r="G93"/>
+      <c r="L93"/>
+      <c r="O93"/>
+    </row>
+    <row r="94" spans="1:16">
+      <c r="C94"/>
+      <c r="F94"/>
+      <c r="G94"/>
+      <c r="L94"/>
+      <c r="O94"/>
+    </row>
+    <row r="95" spans="1:16">
+      <c r="C95"/>
+      <c r="F95"/>
+      <c r="G95"/>
+      <c r="L95"/>
+      <c r="O95"/>
+    </row>
+    <row r="96" spans="1:16">
+      <c r="C96"/>
+      <c r="F96"/>
+      <c r="G96"/>
+      <c r="L96"/>
+      <c r="O96"/>
+    </row>
+    <row r="97" spans="1:16">
+      <c r="C97"/>
+      <c r="F97"/>
+      <c r="G97"/>
+      <c r="L97"/>
+      <c r="O97"/>
+    </row>
+    <row r="98" spans="1:16">
+      <c r="C98"/>
+      <c r="F98"/>
+      <c r="G98"/>
+      <c r="L98"/>
+      <c r="O98"/>
+    </row>
+    <row r="99" spans="1:16">
+      <c r="C99"/>
+      <c r="F99"/>
+      <c r="G99"/>
+      <c r="L99"/>
+      <c r="O99"/>
+    </row>
+    <row r="100" spans="1:16">
+      <c r="C100"/>
+      <c r="F100"/>
+      <c r="G100"/>
+      <c r="L100"/>
+      <c r="O100"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" errorStyle="information" allowBlank="1" sqref="F2:F100" xr:uid="{00000000-0002-0000-0000-000001000000}">
+  <dataValidations count="5">
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" errorTitle="Input Error" error="Prodi tidak ditemukan. Silakan pilih dari dropdown." promptTitle="Pilih Prodi" prompt="Silakan pilih prodi dari dropdown." sqref="C2:C100">
+      <formula1>'Referensi'!$A$1:$A$1</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F2:F100">
       <formula1>"Laki-laki,Perempuan"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="information" allowBlank="1" sqref="G2:G100" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G2:G100">
       <formula1>"Islam,Kristen,Katolik,Hindu,Buddha,Konghucu"</formula1>
     </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" errorTitle="Input Error" error="Status tidak valid. Silakan pilih dari dropdown." promptTitle="Pilih Status Mahasiswa" prompt="Silakan pilih status dari dropdown." sqref="L2:L100">
+      <formula1>'Referensi'!$C$1:$C$5</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" errorTitle="Input Error" error="Gelar tidak ditemukan. Silakan pilih dari dropdown." promptTitle="Pilih Gelar" prompt="Silakan pilih gelar dari dropdown." sqref="O2:O100">
+      <formula1>'Referensi'!$B$1:$B$3</formula1>
+    </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{9626EFD3-ACAA-411A-A201-6B1C0AE0B368}"/>
-  </hyperlinks>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" errorStyle="information" allowBlank="1" errorTitle="Input Error" error="Prodi tidak ditemukan. Silakan pilih dari dropdown." promptTitle="Pilih Prodi" prompt="Silakan pilih prodi dari dropdown." xr:uid="{00000000-0002-0000-0000-000000000000}">
-          <x14:formula1>
-            <xm:f>Referensi!$A$1:$A$1</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C100</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" errorStyle="information" allowBlank="1" errorTitle="Input Error" error="Status tidak valid. Silakan pilih dari dropdown." promptTitle="Pilih Status Mahasiswa" prompt="Silakan pilih status dari dropdown." xr:uid="{00000000-0002-0000-0000-000003000000}">
-          <x14:formula1>
-            <xm:f>Referensi!$C$1:$C$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>L2:L100</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" errorStyle="information" allowBlank="1" errorTitle="Input Error" error="Gelar tidak ditemukan. Silakan pilih dari dropdown." promptTitle="Pilih Gelar" prompt="Silakan pilih gelar dari dropdown." xr:uid="{00000000-0002-0000-0000-000004000000}">
-          <x14:formula1>
-            <xm:f>Referensi!$B$1:$B$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>O2:O100</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:3">
       <c r="B2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="B3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="C4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="C5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>